<commit_message>
Add Media page; drop abstract from 2025 SNAP research letter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pubs/pubs.xlsx
+++ b/pubs/pubs.xlsx
@@ -1,26 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewlavallee/Documents/personal/matthewlavallee.github.io/pubs/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3058862B-B70A-684A-9716-CB79E72A14C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="25440" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="25440" windowHeight="17820" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>authors</t>
   </si>
@@ -192,7 +185,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -229,7 +222,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,11 +518,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -555,11 +548,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>2022</v>
       </c>
       <c r="C2" t="s">
@@ -571,7 +564,7 @@
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="1" t="n">
         <v>44722</v>
       </c>
       <c r="G2" t="s">
@@ -581,11 +574,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>2023</v>
       </c>
       <c r="C3" t="s">
@@ -597,7 +590,7 @@
       <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="1" t="n">
         <v>45147</v>
       </c>
       <c r="G3" t="s">
@@ -607,11 +600,11 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>2024</v>
       </c>
       <c r="C4" t="s">
@@ -623,7 +616,7 @@
       <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="1" t="n">
         <v>45621</v>
       </c>
       <c r="G4" t="s">
@@ -633,11 +626,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5" t="s">
         <v>26</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>2024</v>
       </c>
       <c r="C5" t="s">
@@ -649,7 +642,7 @@
       <c r="E5" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="1" t="n">
         <v>45600</v>
       </c>
       <c r="G5" t="s">
@@ -659,11 +652,11 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="n">
         <v>2026</v>
       </c>
       <c r="C6" t="s">
@@ -672,7 +665,7 @@
       <c r="D6" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="1" t="n">
         <v>46045</v>
       </c>
       <c r="G6" t="s">
@@ -682,11 +675,11 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" t="s">
         <v>35</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="n">
         <v>2026</v>
       </c>
       <c r="C7" t="s">
@@ -695,7 +688,7 @@
       <c r="D7" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="1" t="n">
         <v>46071</v>
       </c>
       <c r="G7" t="s">
@@ -705,11 +698,11 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" t="s">
         <v>40</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="n">
         <v>2025</v>
       </c>
       <c r="C8" t="s">
@@ -718,10 +711,8 @@
       <c r="D8" t="s">
         <v>10</v>
       </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="1">
+      <c r="E8"/>
+      <c r="F8" s="1" t="n">
         <v>45807</v>
       </c>
       <c r="G8" t="s">

</xml_diff>

<commit_message>
Research: per-paper Media dropdown (from pubs.xlsx media column); remove Media page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pubs/pubs.xlsx
+++ b/pubs/pubs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>authors</t>
   </si>
@@ -176,6 +176,13 @@
   </si>
   <si>
     <t>g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Washington Post | March 28, 2026 | Why millions of seniors have suddenly lost health care coverage | https://www.washingtonpost.com/health/2026/03/28/insurance-health-care-medicare-seniors/
+Reuters | February 18, 2026 | Millions of US Medicare Advantage enrollees forced to switch plans, study finds | https://www.reuters.com/legal/litigation/millions-us-medicare-advantage-enrollees-forced-switch-plans-study-finds-2026-02-18/</t>
   </si>
 </sst>
 </file>
@@ -197,7 +204,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -547,6 +553,9 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -696,6 +705,9 @@
       </c>
       <c r="H7" t="s">
         <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="8">

</xml_diff>